<commit_message>
Add bat:warrantyPeriod (xsd:duration), Annex XIII 1(m)
Closes ontologies-core#34.
</commit_message>
<xml_diff>
--- a/Battery_coverage_matrix_issue10.xlsx
+++ b/Battery_coverage_matrix_issue10.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MJELASSI\Downloads\Documents CEA\1-Battery\1-L'ontologie OWL Battery\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CIRPASS\ontologies-battery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEEBF921-1A75-468B-9185-4B710CE5F7D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C247E6F-6A2B-4477-9C46-B9C64DC7B857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Coverage matrix" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="209">
   <si>
     <t>BatteryPass-Ready long list v1.3, attributes 1-100 → CORE term, battery term, or named CORE proposal</t>
   </si>
@@ -660,6 +660,9 @@
   </si>
   <si>
     <t>batloc:BatteryLocationScheme</t>
+  </si>
+  <si>
+    <t>bat:warrantyPeriod</t>
   </si>
 </sst>
 </file>
@@ -1500,11 +1503,12 @@
       <c r="C20" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E20" s="7"/>
-      <c r="F20" s="8"/>
+      <c r="D20" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>208</v>
+      </c>
       <c r="G20" s="12" t="s">
         <v>45</v>
       </c>

</xml_diff>